<commit_message>
mise a jour diagramme
</commit_message>
<xml_diff>
--- a/Diagramme_gantt.xlsx
+++ b/Diagramme_gantt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thomas\Documents\Cours\BUT info\SAE\SAE-2.03\pong\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7BCA2FE-AFE5-4F92-A4C6-E571EC21531F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44EB6840-A5F5-4254-9DB1-6F91A864A272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="600" yWindow="-120" windowWidth="28320" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -677,9 +677,7 @@
       <c r="B9" s="18">
         <v>3</v>
       </c>
-      <c r="C9" s="8">
-        <v>0</v>
-      </c>
+      <c r="C9" s="8"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
@@ -694,9 +692,7 @@
       <c r="B10" s="19">
         <v>1</v>
       </c>
-      <c r="C10" s="8">
-        <v>0</v>
-      </c>
+      <c r="C10" s="8"/>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
       <c r="F10" s="4"/>
@@ -711,9 +707,7 @@
       <c r="B11" s="18">
         <v>1</v>
       </c>
-      <c r="C11" s="8">
-        <v>0</v>
-      </c>
+      <c r="C11" s="8"/>
       <c r="D11" s="4"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -749,7 +743,7 @@
       <c r="F13" s="4"/>
       <c r="G13" s="21"/>
       <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
+      <c r="I13" s="2"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
@@ -764,7 +758,7 @@
       <c r="F14" s="4"/>
       <c r="G14" s="22"/>
       <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
+      <c r="I14" s="3"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">

</xml_diff>

<commit_message>
mise a jour gantt, ajout fichier fonctionnalites
</commit_message>
<xml_diff>
--- a/Diagramme_gantt.xlsx
+++ b/Diagramme_gantt.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thomas\Documents\Cours\BUT info\SAE\SAE-2.03\pong\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ymadr\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44EB6840-A5F5-4254-9DB1-6F91A864A272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{762EFCB0-F2BC-4B1C-818C-0991B1B30692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="600" yWindow="-120" windowWidth="28320" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="34">
   <si>
     <t>tache a réaliser</t>
   </si>
@@ -127,6 +127,18 @@
   </si>
   <si>
     <t>Maintiens git</t>
+  </si>
+  <si>
+    <t>tache à réaliser</t>
+  </si>
+  <si>
+    <t>Les deux</t>
+  </si>
+  <si>
+    <t>Fonctionnalité de base( balle, barre, rebond,score,vies)</t>
+  </si>
+  <si>
+    <t>tester eventuel problème ESP</t>
   </si>
 </sst>
 </file>
@@ -214,7 +226,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF9966FF"/>
+        <fgColor rgb="FF002060"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -269,8 +281,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -294,7 +304,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -585,32 +597,32 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I42"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" style="19" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" style="10" customWidth="1"/>
-    <col min="4" max="9" width="24.85546875" customWidth="1"/>
+    <col min="1" max="1" width="25.33203125" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" style="17" customWidth="1"/>
+    <col min="3" max="3" width="14.88671875" style="10" customWidth="1"/>
+    <col min="4" max="9" width="24.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="15"/>
-    </row>
-    <row r="2" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B1" s="13"/>
+    </row>
+    <row r="2" spans="1:9" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
-      <c r="B2" s="15"/>
-    </row>
-    <row r="3" spans="1:9" s="11" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B2" s="13"/>
+    </row>
+    <row r="3" spans="1:9" s="11" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="18" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="11" t="s">
@@ -623,17 +635,17 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="16"/>
-    </row>
-    <row r="7" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="14"/>
+    </row>
+    <row r="7" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="15" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="7" t="s">
@@ -658,23 +670,23 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A8" s="23" t="s">
+    <row r="8" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="16">
         <v>1</v>
       </c>
       <c r="C8" s="8"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
       <c r="I8" s="1"/>
     </row>
-    <row r="9" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="18">
+      <c r="B9" s="16">
         <v>3</v>
       </c>
       <c r="C9" s="8"/>
@@ -685,11 +697,11 @@
       <c r="H9" s="1"/>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="23" t="s">
+    <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="19">
+      <c r="B10" s="17">
         <v>1</v>
       </c>
       <c r="C10" s="8"/>
@@ -700,84 +712,84 @@
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="18">
+      <c r="B11" s="16">
         <v>1</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="4"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
-      <c r="G11" s="21"/>
+      <c r="G11" s="19"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="18">
+      <c r="B12" s="16">
         <v>3</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="18">
+      <c r="B13" s="16">
         <v>1</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="21"/>
+      <c r="G13" s="19"/>
       <c r="H13" s="4"/>
       <c r="I13" s="2"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="18">
+      <c r="B14" s="16">
         <v>2</v>
       </c>
       <c r="C14" s="8"/>
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="22"/>
+      <c r="G14" s="20"/>
       <c r="H14" s="4"/>
       <c r="I14" s="3"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="18">
+      <c r="B15" s="16">
         <v>1</v>
       </c>
       <c r="C15" s="8"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="24"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="18"/>
+      <c r="B16" s="16"/>
       <c r="C16" s="8"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
@@ -786,9 +798,9 @@
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="18"/>
+      <c r="B17" s="16"/>
       <c r="C17" s="8"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
@@ -797,9 +809,9 @@
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="18"/>
+      <c r="B18" s="16"/>
       <c r="C18" s="8"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
@@ -808,10 +820,10 @@
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C19" s="9"/>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C21" s="10" t="s">
         <v>11</v>
       </c>
@@ -821,11 +833,11 @@
       <c r="E21" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F21" s="14" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F21" s="22" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D22" t="s">
         <v>20</v>
       </c>
@@ -833,17 +845,17 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B25" s="16"/>
-    </row>
-    <row r="27" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="14"/>
+    </row>
+    <row r="27" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B27" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="15" t="s">
         <v>15</v>
       </c>
       <c r="C27" s="7" t="s">
@@ -868,97 +880,144 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="1"/>
-      <c r="B28" s="18"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="1"/>
-      <c r="B29" s="18"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="21"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="1"/>
-      <c r="B30" s="18"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="1"/>
-      <c r="B31" s="18"/>
-      <c r="C31" s="8"/>
+    <row r="28" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="16">
+        <v>1</v>
+      </c>
+      <c r="C28" s="8">
+        <v>1</v>
+      </c>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="I28" s="1"/>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B29" s="16">
+        <v>3</v>
+      </c>
+      <c r="C29" s="8">
+        <v>1</v>
+      </c>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+    </row>
+    <row r="30" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A30" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="17">
+        <v>1</v>
+      </c>
+      <c r="C30" s="8">
+        <v>0.85</v>
+      </c>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31" s="16">
+        <v>1</v>
+      </c>
+      <c r="C31" s="8">
+        <v>0.8</v>
+      </c>
       <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="1"/>
-      <c r="B32" s="18"/>
-      <c r="C32" s="8"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="2"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B32" s="16">
+        <v>3</v>
+      </c>
+      <c r="C32" s="8">
+        <v>0.9</v>
+      </c>
       <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="22"/>
-      <c r="H32" s="22"/>
-      <c r="I32" s="4"/>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="1"/>
-      <c r="B33" s="18"/>
-      <c r="C33" s="8"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="23"/>
+      <c r="I32" s="23"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B33" s="16">
+        <v>1</v>
+      </c>
+      <c r="C33" s="8">
+        <v>0.25</v>
+      </c>
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
-      <c r="G33" s="22"/>
+      <c r="G33" s="19"/>
       <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="1"/>
-      <c r="B34" s="18"/>
-      <c r="C34" s="8"/>
+      <c r="I33" s="2"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B34" s="16">
+        <v>2</v>
+      </c>
+      <c r="C34" s="8">
+        <v>1</v>
+      </c>
       <c r="D34" s="4"/>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="1"/>
-      <c r="B35" s="18"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
-      <c r="I35" s="4"/>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="1"/>
-      <c r="B36" s="18"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="2"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" s="16">
+        <v>1</v>
+      </c>
+      <c r="C35" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="D35" s="3"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="24"/>
+      <c r="I35" s="24"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A36" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B36" s="16"/>
       <c r="C36" s="8"/>
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
@@ -967,9 +1026,9 @@
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
-      <c r="B37" s="18"/>
+      <c r="B37" s="16"/>
       <c r="C37" s="8"/>
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
@@ -978,9 +1037,9 @@
       <c r="H37" s="4"/>
       <c r="I37" s="4"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
-      <c r="B38" s="18"/>
+      <c r="B38" s="16"/>
       <c r="C38" s="8"/>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
@@ -989,10 +1048,10 @@
       <c r="H38" s="4"/>
       <c r="I38" s="4"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C39" s="9"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C41" s="10" t="s">
         <v>11</v>
       </c>
@@ -1002,11 +1061,11 @@
       <c r="E41" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F41" s="14" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F41" s="22" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="D42" t="s">
         <v>20</v>
       </c>

</xml_diff>